<commit_message>
add 541 ex questions
</commit_message>
<xml_diff>
--- a/ids541_specific/class_schedule_541_xlsx.xlsx
+++ b/ids541_specific/class_schedule_541_xlsx.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nce8/github/practicaldatascience_book/ids541_specific/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBB508ED-1889-4E45-BCAE-853DD047A4CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{286C865F-8841-EB41-A5B7-444EAEEC9AE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17260" xr2:uid="{212B26BE-C12B-1745-A277-D3917F547107}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="83">
   <si>
     <t>Topic</t>
   </si>
@@ -311,6 +311,9 @@
   </si>
   <si>
     <t>- `Answering Questions (include inference/prediction comparison) &lt;https://ds4humans.com/30_questions/00_solving_problems_by_answering_questions.html&gt;`_</t>
+  </si>
+  <si>
+    <t>`Questions Ex &lt;https://ds4humans.com/99_exercises/exercise_probs_and_questions.html&gt;`_</t>
   </si>
 </sst>
 </file>
@@ -951,7 +954,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>40</v>
       </c>
@@ -960,6 +963,9 @@
       </c>
       <c r="C21" s="9" t="s">
         <v>81</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="106" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>